<commit_message>
Judge v1 results: agreement 46%, kappa 0.14
</commit_message>
<xml_diff>
--- a/data/judge_sample.xlsx
+++ b/data/judge_sample.xlsx
@@ -1,33 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\abdiddoj\project1\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D5AC069-BFC3-4E12-A937-8333617DD9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="judge_sample" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="135">
   <si>
     <t>item_id</t>
   </si>
@@ -77,7 +70,7 @@
     <t>POOL0613</t>
   </si>
   <si>
-    <t>Flexing their cars ??</t>
+    <t>Flexing their cars 🚗</t>
   </si>
   <si>
     <t>Hate Speech</t>
@@ -101,7 +94,7 @@
     <t>POOL0573</t>
   </si>
   <si>
-    <t>1h walking to the house ????</t>
+    <t>1h walking to the house 💔🥲</t>
   </si>
   <si>
     <t>No hateful content, but no other category fits</t>
@@ -128,7 +121,7 @@
     <t>POOL0411</t>
   </si>
   <si>
-    <t>??? 1998 winkom blhy raw whd bch yehbl</t>
+    <t>جيل 1998 winkom blhy raw whd bch yehbl</t>
   </si>
   <si>
     <t>The comment appears to be a playful, nonsensical phrase typical of humorous or teasing remarks in Tunisian Darija, with no clear hateful or positive content.</t>
@@ -158,16 +151,16 @@
     <t>POOL0005</t>
   </si>
   <si>
-    <t>Let him be, it's the dragon of dirge ????</t>
-  </si>
-  <si>
-    <t>The comment uses a playful exaggeration (dragon of dirge) and crying emojis, indicating a humorous or ironic tone rather than praise or hate.</t>
+    <t>Let him be, it's the dragon of dirge 😭😭</t>
+  </si>
+  <si>
+    <t>The comment uses a playful exaggeration (“dragon of dirge”) and crying emojis, indicating a humorous or ironic tone rather than praise or hate.</t>
   </si>
   <si>
     <t>POOL0202</t>
   </si>
   <si>
-    <t>@user walla ahebek??????</t>
+    <t>@user walla ahebek🥹😘😘</t>
   </si>
   <si>
     <t>Expresses affection and love with emojis</t>
@@ -179,7 +172,7 @@
     <t>POOL0464</t>
   </si>
   <si>
-    <t>?Kberet f lac residence bl acenseur ?</t>
+    <t>✨Kberet f lac residence bl acenseur ✨</t>
   </si>
   <si>
     <t>The comment praises the growth or improvement of the residence, indicating a positive reaction.</t>
@@ -188,7 +181,7 @@
     <t>POOL0154</t>
   </si>
   <si>
-    <t>@user handcream and sunscreen fs??????</t>
+    <t>@user handcream and sunscreen fs😭🫶🏻</t>
   </si>
   <si>
     <t>The comment recommends hand cream and sunscreen, expressing a supportive or appreciative stance toward the product.</t>
@@ -197,7 +190,7 @@
     <t>POOL0353</t>
   </si>
   <si>
-    <t>Omgggg youu killed meeee ????????????</t>
+    <t>Omgggg youu killed meeee 🤣🤣🤣🤣🤣🤣</t>
   </si>
   <si>
     <t>The comment expresses amusement with laughing emojis, indicating a playful, humorous reaction.</t>
@@ -215,7 +208,7 @@
     <t>POOL0374</t>
   </si>
   <si>
-    <t>Casual msb student??????????</t>
+    <t>Casual msb student🤌🏻😂😂😂</t>
   </si>
   <si>
     <t>The comment uses laughing emojis and a playful phrase that appears to be a joke rather than a genuine compliment or hateful content.</t>
@@ -233,7 +226,7 @@
     <t>POOL0567</t>
   </si>
   <si>
-    <t>Pov: camera man??</t>
+    <t>Pov: camera man😢</t>
   </si>
   <si>
     <t>The comment is neutral and not hateful; it does not express positive praise or humor, but it is not hateful, so the closest category is Humour.</t>
@@ -242,7 +235,7 @@
     <t>POOL0231</t>
   </si>
   <si>
-    <t>@user ???? ? ??? ????</t>
+    <t>@user ركزي ع اول وحده</t>
   </si>
   <si>
     <t>Encouraging directive to focus on the first person</t>
@@ -251,7 +244,7 @@
     <t>POOL0373</t>
   </si>
   <si>
-    <t>Hetou chwaya????</t>
+    <t>Hetou chwaya😢😢</t>
   </si>
   <si>
     <t>Neutral comment, not hateful or positive, so default to Humour</t>
@@ -260,7 +253,7 @@
     <t>POOL0140</t>
   </si>
   <si>
-    <t>@user buy me the mist please ??</t>
+    <t>@user buy me the mist please 😭</t>
   </si>
   <si>
     <t>The comment is a playful request and does not contain hate speech, so it is classified as Humour.</t>
@@ -269,7 +262,7 @@
     <t>POOL0161</t>
   </si>
   <si>
-    <t>@user my soulmate ??</t>
+    <t>@user my soulmate ❤️</t>
   </si>
   <si>
     <t>expresses affection and admiration</t>
@@ -278,7 +271,7 @@
     <t>POOL0390</t>
   </si>
   <si>
-    <t>they have to be doing jt on purpose ??</t>
+    <t>they have to be doing jt on purpose 😂</t>
   </si>
   <si>
     <t>The comment is a playful joke with a laughing emoji, not praising or hateful.</t>
@@ -305,16 +298,16 @@
     <t>POOL0016</t>
   </si>
   <si>
-    <t>@user ???????? nahna</t>
-  </si>
-  <si>
-    <t>The comment uses laughing emojis and a short, non?offensive word, indicating a playful or humorous tone rather than praise or hate.</t>
+    <t>@user 😂😂😂😂 nahna</t>
+  </si>
+  <si>
+    <t>The comment uses laughing emojis and a short, non‑offensive word, indicating a playful or humorous tone rather than praise or hate.</t>
   </si>
   <si>
     <t>POOL0593</t>
   </si>
   <si>
-    <t>??? ??? ??? ???? (????? ?????)</t>
+    <t>هاي هاي على رونج (هلكني الحسد)</t>
   </si>
   <si>
     <t>The comment expresses excitement and admiration, indicating a positive reaction to the content.</t>
@@ -323,7 +316,7 @@
     <t>POOL0226</t>
   </si>
   <si>
-    <t>@user ??????</t>
+    <t>@user قلبم💗</t>
   </si>
   <si>
     <t>The comment expresses affection with a heart emoji, indicating a positive reaction.</t>
@@ -332,7 +325,7 @@
     <t>POOL0234</t>
   </si>
   <si>
-    <t>Personal hotspot ????</t>
+    <t>Personal hotspot 🫂💗</t>
   </si>
   <si>
     <t>The comment expresses affection and support with emojis, indicating a positive reaction.</t>
@@ -359,7 +352,7 @@
     <t>POOL0352</t>
   </si>
   <si>
-    <t>The best duo??????</t>
+    <t>The best duo🤌🏻😂</t>
   </si>
   <si>
     <t>Expresses praise and appreciation for the duo</t>
@@ -386,8 +379,8 @@
     <t>POOL0201</t>
   </si>
   <si>
-    <t>My darlings???? @user &amp; @user 
-I love u guys????</t>
+    <t>My darlings🥹❤️ @user &amp; @user 
+I love u guys❤️🫂</t>
   </si>
   <si>
     <t>Expresses affection and love toward the users.</t>
@@ -396,13 +389,13 @@
     <t>POOL0262</t>
   </si>
   <si>
-    <t>@user girllll??????</t>
+    <t>@user girllll😂😂💗</t>
   </si>
   <si>
     <t>POOL0006</t>
   </si>
   <si>
-    <t>@user ???? ?????? ????????</t>
+    <t>@user ماذا يفعلون فالمعبد؟</t>
   </si>
   <si>
     <t>Neutral question, not hateful or humorous</t>
@@ -411,7 +404,7 @@
     <t>POOL0363</t>
   </si>
   <si>
-    <t>HAHAHAHAHA ??????</t>
+    <t>HAHAHAHAHA 😂😂😂</t>
   </si>
   <si>
     <t>laughing expression</t>
@@ -420,7 +413,7 @@
     <t>POOL0157</t>
   </si>
   <si>
-    <t>@user ????real especially the hand cream</t>
+    <t>@user 😩😩real especially the hand cream</t>
   </si>
   <si>
     <t>Ambiguous, not hateful, no clear positivity.</t>
@@ -429,23 +422,17 @@
     <t>POOL0513</t>
   </si>
   <si>
-    <t>??? ?????</t>
-  </si>
-  <si>
-    <t>The comment contains the insulting word "?????" (snot/boogers), which is a derogatory term used to insult someone.</t>
+    <t>جيل خنانة</t>
+  </si>
+  <si>
+    <t>The comment contains the insulting word "خنانة" (snot/boogers), which is a derogatory term used to insult someone.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -453,346 +440,16 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -800,345 +457,173 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -1149,7 +634,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1177,154 +662,40 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1582,19 +953,19 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H41"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="46.4444444444444" customWidth="1"/>
-    <col min="3" max="3" width="15.3333333333333" customWidth="1"/>
-    <col min="5" max="5" width="124.333333333333" customWidth="1"/>
-    <col min="6" max="6" width="9.55555555555556" customWidth="1"/>
+    <col min="2" max="2" width="46.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="124.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.5546875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1643,7 +1014,10 @@
         <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1668,6 +1042,9 @@
       <c r="G3" t="s">
         <v>19</v>
       </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
@@ -1691,6 +1068,9 @@
       <c r="G4" t="s">
         <v>19</v>
       </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
@@ -1712,7 +1092,10 @@
         <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>19</v>
+      </c>
+      <c r="H5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1737,6 +1120,9 @@
       <c r="G6" t="s">
         <v>14</v>
       </c>
+      <c r="H6" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
@@ -1755,10 +1141,13 @@
         <v>31</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7" t="s">
-        <v>14</v>
+        <v>19</v>
+      </c>
+      <c r="H7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1783,6 +1172,9 @@
       <c r="G8" t="s">
         <v>14</v>
       </c>
+      <c r="H8" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
@@ -1804,7 +1196,10 @@
         <v>13</v>
       </c>
       <c r="G9" t="s">
-        <v>14</v>
+        <v>19</v>
+      </c>
+      <c r="H9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1829,6 +1224,9 @@
       <c r="G10" t="s">
         <v>14</v>
       </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
@@ -1852,6 +1250,9 @@
       <c r="G11" t="s">
         <v>14</v>
       </c>
+      <c r="H11" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
@@ -1875,6 +1276,9 @@
       <c r="G12" t="s">
         <v>35</v>
       </c>
+      <c r="H12" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
@@ -1898,6 +1302,9 @@
       <c r="G13" t="s">
         <v>19</v>
       </c>
+      <c r="H13" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
@@ -1921,6 +1328,9 @@
       <c r="G14" t="s">
         <v>14</v>
       </c>
+      <c r="H14" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
@@ -1942,7 +1352,10 @@
         <v>13</v>
       </c>
       <c r="G15" t="s">
-        <v>14</v>
+        <v>19</v>
+      </c>
+      <c r="H15" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1965,10 +1378,13 @@
         <v>13</v>
       </c>
       <c r="G16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
         <v>61</v>
       </c>
@@ -1988,10 +1404,13 @@
         <v>13</v>
       </c>
       <c r="G17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
         <v>64</v>
       </c>
@@ -2013,8 +1432,11 @@
       <c r="G18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="H18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
         <v>67</v>
       </c>
@@ -2036,8 +1458,11 @@
       <c r="G19" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="H19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
         <v>70</v>
       </c>
@@ -2059,8 +1484,11 @@
       <c r="G20" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="H20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -2082,8 +1510,11 @@
       <c r="G21" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="H21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
         <v>76</v>
       </c>
@@ -2100,13 +1531,16 @@
         <v>78</v>
       </c>
       <c r="F22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G22" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" t="s">
         <v>79</v>
       </c>
@@ -2128,8 +1562,11 @@
       <c r="G23" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="H23" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" t="s">
         <v>82</v>
       </c>
@@ -2151,8 +1588,11 @@
       <c r="G24" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="H24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
         <v>85</v>
       </c>
@@ -2172,10 +1612,13 @@
         <v>13</v>
       </c>
       <c r="G25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" t="s">
         <v>88</v>
       </c>
@@ -2195,10 +1638,13 @@
         <v>13</v>
       </c>
       <c r="G26" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" t="s">
         <v>91</v>
       </c>
@@ -2218,10 +1664,13 @@
         <v>13</v>
       </c>
       <c r="G27" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" t="s">
         <v>94</v>
       </c>
@@ -2241,10 +1690,13 @@
         <v>13</v>
       </c>
       <c r="G28" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H28" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" t="s">
         <v>97</v>
       </c>
@@ -2266,8 +1718,11 @@
       <c r="G29" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="H29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" t="s">
         <v>100</v>
       </c>
@@ -2287,10 +1742,13 @@
         <v>13</v>
       </c>
       <c r="G30" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H30" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" t="s">
         <v>103</v>
       </c>
@@ -2310,10 +1768,13 @@
         <v>13</v>
       </c>
       <c r="G31" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H31" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" t="s">
         <v>106</v>
       </c>
@@ -2335,8 +1796,11 @@
       <c r="G32" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="33" spans="1:7">
+      <c r="H32" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
         <v>109</v>
       </c>
@@ -2356,10 +1820,13 @@
         <v>13</v>
       </c>
       <c r="G33" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H33" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" t="s">
         <v>112</v>
       </c>
@@ -2381,8 +1848,11 @@
       <c r="G34" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="35" spans="1:7">
+      <c r="H34" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
         <v>115</v>
       </c>
@@ -2404,8 +1874,11 @@
       <c r="G35" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="36" ht="86.4" spans="1:7">
+      <c r="H35" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="28.8" customHeight="1">
       <c r="A36" t="s">
         <v>118</v>
       </c>
@@ -2427,8 +1900,11 @@
       <c r="G36" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="37" spans="1:7">
+      <c r="H36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" t="s">
         <v>121</v>
       </c>
@@ -2450,8 +1926,11 @@
       <c r="G37" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="38" spans="1:7">
+      <c r="H37" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" t="s">
         <v>123</v>
       </c>
@@ -2468,13 +1947,16 @@
         <v>125</v>
       </c>
       <c r="F38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G38" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H38" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" t="s">
         <v>126</v>
       </c>
@@ -2491,13 +1973,16 @@
         <v>128</v>
       </c>
       <c r="F39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G39" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+        <v>19</v>
+      </c>
+      <c r="H39" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" t="s">
         <v>129</v>
       </c>
@@ -2519,8 +2004,11 @@
       <c r="G40" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="41" spans="1:7">
+      <c r="H40" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" t="s">
         <v>132</v>
       </c>
@@ -2542,14 +2030,16 @@
       <c r="G41" t="s">
         <v>14</v>
       </c>
+      <c r="H41" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F41">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F41" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"good ,bad ,partly"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>